<commit_message>
vault backup: 2026-09-19 22:37:43
</commit_message>
<xml_diff>
--- a/01-Projects/에이팜건강-주간자금계획-자동화/자금계획_자동화/02_경영지원_대외비/지출계획_2026-09-19.xlsx
+++ b/01-Projects/에이팜건강-주간자금계획-자동화/자금계획_자동화/02_경영지원_대외비/지출계획_2026-09-19.xlsx
@@ -1063,22 +1063,22 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>건강-20260918-005</t>
+          <t>경영-20260918-015</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>건강</t>
+          <t>경영</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>건강사업팀</t>
+          <t>경영지원팀</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>전은신</t>
+          <t>김정원</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1087,25 +1087,25 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>써치엠</t>
+          <t>엠에스바이오텍</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>메타 광고 대행 수수</t>
+          <t>외상매입금</t>
         </is>
       </c>
       <c r="J10" s="2" t="n">
-        <v>1487786</v>
+        <v>20000000</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -1114,24 +1114,29 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>신규</t>
+          <t>변경</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>8월 광고비에 대한 수수료 11%</t>
+          <t>외상매입금 1차 지급</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>기타 대외비 지출</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>건강-20260918-006</t>
+          <t>건강-20260918-005</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1155,7 +1160,7 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -1164,16 +1169,16 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>네이버SA&amp;GFA</t>
+          <t>써치엠</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>네이버SA&amp;GFA 광고 비용 충전</t>
+          <t>메타 광고 대행 수수</t>
         </is>
       </c>
       <c r="J11" s="2" t="n">
-        <v>8305000</v>
+        <v>1487786</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -1192,14 +1197,14 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>금주 목~차주 월까지 광고비 충전 금액</t>
+          <t>8월 광고비에 대한 수수료 11%</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>건강-20260918-007</t>
+          <t>건강-20260918-006</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1223,7 +1228,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -1232,16 +1237,16 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>ADN</t>
+          <t>네이버SA&amp;GFA</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>ADN 광고-추석 유입</t>
+          <t>네이버SA&amp;GFA 광고 비용 충전</t>
         </is>
       </c>
       <c r="J12" s="2" t="n">
-        <v>550000</v>
+        <v>8305000</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
@@ -1256,28 +1261,33 @@
       <c r="N12" t="inlineStr">
         <is>
           <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>금주 목~차주 월까지 광고비 충전 금액</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>경영-20260918-003</t>
+          <t>건강-20260918-007</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>경영</t>
+          <t>건강</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>경영지원팀</t>
+          <t>건강사업팀</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>김수희</t>
+          <t>전은신</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1286,7 +1296,7 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -1295,20 +1305,20 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>농협카드</t>
+          <t>ADN</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>8월 카드대금</t>
+          <t>ADN 광고-추석 유입</t>
         </is>
       </c>
       <c r="J13" s="2" t="n">
-        <v>6827883</v>
+        <v>550000</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>자동이체</t>
+          <t>계좌송금</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1319,18 +1329,13 @@
       <c r="N13" t="inlineStr">
         <is>
           <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>기타 대외비 지출</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>경영-20260918-004</t>
+          <t>경영-20260918-003</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1354,7 +1359,7 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -1363,16 +1368,16 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>우리카드</t>
+          <t>농협카드</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>8월 우리카드 카드대금</t>
+          <t>8월 카드대금</t>
         </is>
       </c>
       <c r="J14" s="2" t="n">
-        <v>25346349</v>
+        <v>6827883</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
@@ -1398,7 +1403,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>경영-20260918-012</t>
+          <t>경영-20260918-004</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1413,7 +1418,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>송채은</t>
+          <t>김수희</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1422,7 +1427,7 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1431,20 +1436,20 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>비씨카드</t>
+          <t>우리카드</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>8월카드대금</t>
+          <t>8월 우리카드 카드대금</t>
         </is>
       </c>
       <c r="J15" s="2" t="n">
-        <v>269810</v>
+        <v>25346349</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>계좌송금</t>
+          <t>자동이체</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1457,16 +1462,16 @@
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>에이팜</t>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>기타 대외비 지출</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>경영-20260918-015</t>
+          <t>경영-20260918-012</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1481,7 +1486,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>김정원</t>
+          <t>송채은</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1490,7 +1495,7 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1499,16 +1504,16 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>엠에스바이오텍</t>
+          <t>비씨카드</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>외상매입금</t>
+          <t>8월카드대금</t>
         </is>
       </c>
       <c r="J16" s="2" t="n">
-        <v>20000000</v>
+        <v>269810</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -1517,22 +1522,17 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>변경</t>
+          <t>신규</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>외상매입금 1차 지급</t>
-        </is>
-      </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>기타 대외비 지출</t>
+          <t>에이팜</t>
         </is>
       </c>
     </row>

</xml_diff>